<commit_message>
Actualiza la documentacion con el cierre de NC-001 y NC-008
- Plan de pruebas version 2.3: bitacora (NC-001 y NC-008 cerradas el
  15/10/2026 tras la prueba de confirmacion), estado de los casos CP-004
  y CP-005, arquitectura, OWASP, riesgos (R01 baja a nivel medio) y
  conclusiones.
- Excel GA9-AA2-EV01: NC-001 cerrada en Seguimiento y en la matriz resumen.
- Guia conceptual y curso: estado actualizado; el curso pasa a
  "Archivos de estudio" junto al resto del material.
- herramientas/md2docx.js: conversor del plan de Markdown a Word (APA 7).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Documentacion/GA9/GA9-220501096-AA2-EV01_Casos_Prueba_PetConnect.xlsx
+++ b/Documentacion/GA9/GA9-220501096-AA2-EV01_Casos_Prueba_PetConnect.xlsx
@@ -5,13 +5,13 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\goku8\OneDrive\Escritorio\Evidecia\Documentacion\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\goku8\OneDrive\Escritorio\Evidecia\Documentacion\GA9\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{15AE1F3A-2E3A-4710-854E-3DD248296F51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7CBC5AE5-0A6E-4D6F-9D6B-D76F6A25878F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection lockStructure="1"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4665" yWindow="2670" windowWidth="21600" windowHeight="11835" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info Proyecto" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="594" uniqueCount="354">
   <si>
     <t>FORMATO DE CASOS DE PRUEBA DE SOFTWARE</t>
   </si>
@@ -698,9 +698,6 @@
     <t>Fecha Resolución</t>
   </si>
   <si>
-    <t>Las contraseñas se guardan con SHA-256 sin sal (api.py, función _hash_password): el hash coincide con el SHA-256 de la contraseña y es idéntico entre usuarios. Corrección: bcrypt con costo 12 y migración de los hashes existentes.</t>
-  </si>
-  <si>
     <t>Pendiente</t>
   </si>
   <si>
@@ -1085,10 +1082,22 @@
     <t>Camilo Orjuela y Jazmín Bautista (confirmación: Daniel Jiménez)</t>
   </si>
   <si>
-    <t>Nota: la plantilla tiene tres niveles de severidad (Alta, Media, Baja). NC-001, que el plan de pruebas clasifica como crítica, se registra aquí como Alta. Códigos y severidades coinciden con la bitácora del plan GA9-220501096-AA1-EV02 (versión 2.2).</t>
-  </si>
-  <si>
     <t>Con 500 usuarios, p95 de 30 s y 56 % de errores. La conexión única a la base de datos (Singleton) compartida entre hilos se corrompe ('MySQL Connection not available', 'bytearray index out of range'). Corrección: pool de conexiones, paginación y Gunicorn.</t>
+  </si>
+  <si>
+    <t>Las contraseñas se guardan con SHA-256 sin sal (api.py, función _hash_password): el hash coincide con el SHA-256 de la contraseña y es idéntico entre usuarios. Corrección: bcrypt con costo 12 y migración de los hashes existentes. Corregida y confirmada el 15/10/2026 (Documentacion/Evidencias-Confirmacion-NC-001-NC-008).</t>
+  </si>
+  <si>
+    <t>Cerrado</t>
+  </si>
+  <si>
+    <t>15/10/2026 (prueba de confirmación aprobada)</t>
+  </si>
+  <si>
+    <t>Nota: la plantilla tiene tres niveles de severidad (Alta, Media, Baja). NC-001, que el plan de pruebas clasifica como crítica, se registra aquí como Alta. Códigos y severidades coinciden con la bitácora del plan GA9-220501096-AA1-EV02 (versión 2.3).</t>
+  </si>
+  <si>
+    <t>Cerrado (15/10/2026)</t>
   </si>
 </sst>
 </file>
@@ -1098,7 +1107,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1247,8 +1256,22 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FF059669"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF059669"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="15">
+  <fills count="16">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1330,6 +1353,12 @@
         <fgColor rgb="FF1B2A4A"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDCFCE7"/>
+        <bgColor rgb="FFFEF3C7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="5">
     <border>
@@ -1391,7 +1420,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -1534,6 +1563,12 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2981,7 +3016,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="60" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>164</v>
       </c>
@@ -2989,22 +3024,22 @@
         <v>157</v>
       </c>
       <c r="C3" s="5" t="s">
-        <v>220</v>
+        <v>349</v>
       </c>
       <c r="D3" s="17" t="s">
         <v>154</v>
       </c>
       <c r="E3" s="7" t="s">
-        <v>348</v>
-      </c>
-      <c r="F3" s="13" t="s">
-        <v>221</v>
+        <v>347</v>
+      </c>
+      <c r="F3" s="52" t="s">
+        <v>350</v>
       </c>
       <c r="G3" s="24">
         <v>46300</v>
       </c>
       <c r="H3" s="7" t="s">
-        <v>222</v>
+        <v>351</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="66.400000000000006" customHeight="1" x14ac:dyDescent="0.25">
@@ -3015,7 +3050,7 @@
         <v>146</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="D4" s="12" t="s">
         <v>154</v>
@@ -3024,13 +3059,13 @@
         <v>96</v>
       </c>
       <c r="F4" s="13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G4" s="22">
         <v>46300</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="66.400000000000006" customHeight="1" x14ac:dyDescent="0.25">
@@ -3041,22 +3076,22 @@
         <v>167</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="D5" s="17" t="s">
         <v>154</v>
       </c>
       <c r="E5" s="7" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="F5" s="13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G5" s="24">
         <v>46300</v>
       </c>
       <c r="H5" s="7" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
     </row>
     <row r="6" spans="1:8" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3067,33 +3102,33 @@
         <v>104</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="D6" s="14" t="s">
         <v>112</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F6" s="13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G6" s="22">
         <v>46300</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="81" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>229</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="C7" s="5" t="s">
         <v>230</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>231</v>
       </c>
       <c r="D7" s="17" t="s">
         <v>154</v>
@@ -3102,13 +3137,13 @@
         <v>96</v>
       </c>
       <c r="F7" s="13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G7" s="24">
         <v>46300</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="81" customHeight="1" x14ac:dyDescent="0.25">
@@ -3119,7 +3154,7 @@
         <v>201</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>154</v>
@@ -3128,13 +3163,13 @@
         <v>96</v>
       </c>
       <c r="F8" s="13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G8" s="22">
         <v>46300</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="60" x14ac:dyDescent="0.25">
@@ -3145,22 +3180,22 @@
         <v>125</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="D9" s="15" t="s">
         <v>112</v>
       </c>
       <c r="E9" s="7" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="F9" s="13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G9" s="24">
         <v>46300</v>
       </c>
       <c r="H9" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3171,7 +3206,7 @@
         <v>135</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D10" s="16" t="s">
         <v>143</v>
@@ -3180,18 +3215,18 @@
         <v>96</v>
       </c>
       <c r="F10" s="13" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G10" s="22">
         <v>46300</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="41" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="B12" s="42"/>
       <c r="C12" s="42"/>
@@ -3233,7 +3268,7 @@
   <sheetData>
     <row r="1" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="43" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B1" s="35"/>
       <c r="C1" s="35"/>
@@ -3241,7 +3276,7 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B2" s="18">
         <f>COUNTA('Casos de Prueba'!A3:A14)</f>
@@ -3250,7 +3285,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B3" s="19">
         <f>COUNTIF('Casos de Prueba'!K3:K14,"Aprobado")</f>
@@ -3268,7 +3303,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B5" s="21">
         <f>COUNTIF('Casos de Prueba'!K3:K14,"Rechazado")</f>
@@ -3277,7 +3312,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B6" s="18">
         <f>COUNTA('Casos de Prueba'!K3:K14)</f>
@@ -3286,7 +3321,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B7" s="18">
         <f>COUNTIF('Casos de Prueba'!M3:M14,"Alta")</f>
@@ -3295,7 +3330,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B8" s="18">
         <f>COUNTIF('Casos de Prueba'!M3:M14,"Media")</f>
@@ -3304,7 +3339,7 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B9" s="18">
         <f>COUNTIF('Casos de Prueba'!M3:M14,"Baja")</f>
@@ -3313,7 +3348,7 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B10" s="18">
         <f>COUNTIF(Seguimiento!A3:A20,"NC-*")</f>
@@ -3322,7 +3357,7 @@
     </row>
     <row r="11" spans="1:4" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B11" s="26">
         <f>IF(B2=0,0,B3/B2)</f>
@@ -3331,16 +3366,16 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B12" s="18">
         <f>COUNTIFS(Seguimiento!A3:A20,"NC-*",Seguimiento!F3:F20,"&lt;&gt;Cerrado")</f>
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="49" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B13" s="35"/>
       <c r="C13" s="35"/>
@@ -3348,7 +3383,7 @@
     </row>
     <row r="15" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="47" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B15" s="35"/>
       <c r="C15" s="35"/>
@@ -3356,27 +3391,27 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="44" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B17" s="35"/>
       <c r="C17" s="48" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="D17" s="46"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="44" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="B19" s="35"/>
       <c r="C19" s="46" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="D19" s="46"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="44" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="B21" s="35"/>
       <c r="C21" s="45">
@@ -3418,7 +3453,7 @@
   <sheetData>
     <row r="1" spans="1:5" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="50" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="B1" s="35"/>
       <c r="C1" s="35"/>
@@ -3427,44 +3462,44 @@
     </row>
     <row r="2" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>253</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>254</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="C2" s="6" t="s">
         <v>255</v>
-      </c>
-      <c r="C2" s="6" t="s">
-        <v>256</v>
       </c>
       <c r="D2" s="6" t="s">
         <v>217</v>
       </c>
       <c r="E2" s="6" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="37.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="B3" s="5" t="s">
         <v>258</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="C3" s="5" t="s">
         <v>259</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>260</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>110</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="B4" s="10" t="s">
         <v>262</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>263</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>115</v>
@@ -3473,7 +3508,7 @@
         <v>99</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3481,24 +3516,24 @@
         <v>134</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>265</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>266</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>110</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
     </row>
     <row r="6" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>268</v>
-      </c>
-      <c r="B6" s="10" t="s">
-        <v>269</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>115</v>
@@ -3507,24 +3542,24 @@
         <v>99</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="7" spans="1:5" ht="37.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
+        <v>270</v>
+      </c>
+      <c r="B7" s="5" t="s">
         <v>271</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="C7" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="D7" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="E7" s="5" t="s">
         <v>272</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>270</v>
-      </c>
-      <c r="D7" s="27" t="s">
-        <v>221</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>273</v>
       </c>
     </row>
     <row r="8" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3532,7 +3567,7 @@
         <v>145</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>135</v>
@@ -3541,41 +3576,41 @@
         <v>110</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="9" spans="1:5" ht="37.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="B9" s="5" t="s">
         <v>276</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="C9" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="D9" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>277</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>270</v>
-      </c>
-      <c r="D9" s="27" t="s">
-        <v>221</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>278</v>
       </c>
     </row>
     <row r="10" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="9" t="s">
+        <v>278</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>279</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="C10" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="D10" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="E10" s="10" t="s">
         <v>280</v>
-      </c>
-      <c r="C10" s="10" t="s">
-        <v>270</v>
-      </c>
-      <c r="D10" s="27" t="s">
-        <v>221</v>
-      </c>
-      <c r="E10" s="10" t="s">
-        <v>281</v>
       </c>
     </row>
     <row r="11" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
@@ -3583,7 +3618,7 @@
         <v>211</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>201</v>
@@ -3592,171 +3627,171 @@
         <v>152</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="9" t="s">
+        <v>283</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>284</v>
       </c>
-      <c r="B12" s="10" t="s">
+      <c r="C12" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="D12" s="28" t="s">
         <v>285</v>
       </c>
-      <c r="C12" s="10" t="s">
-        <v>270</v>
-      </c>
-      <c r="D12" s="28" t="s">
+      <c r="E12" s="10" t="s">
         <v>286</v>
-      </c>
-      <c r="E12" s="10" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="13" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
+        <v>287</v>
+      </c>
+      <c r="B13" s="5" t="s">
         <v>288</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>289</v>
-      </c>
       <c r="C13" s="5" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D13" s="28" t="s">
+        <v>285</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>286</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>287</v>
       </c>
     </row>
     <row r="14" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="9" t="s">
+        <v>289</v>
+      </c>
+      <c r="B14" s="10" t="s">
         <v>290</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="C14" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="D14" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="E14" s="10" t="s">
         <v>291</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>270</v>
-      </c>
-      <c r="D14" s="27" t="s">
-        <v>221</v>
-      </c>
-      <c r="E14" s="10" t="s">
-        <v>292</v>
       </c>
     </row>
     <row r="15" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
+        <v>292</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>293</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="C15" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="D15" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="E15" s="5" t="s">
         <v>294</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>270</v>
-      </c>
-      <c r="D15" s="27" t="s">
-        <v>221</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="16" spans="1:5" ht="37.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="9" t="s">
+        <v>295</v>
+      </c>
+      <c r="B16" s="10" t="s">
         <v>296</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="C16" s="10" t="s">
         <v>297</v>
-      </c>
-      <c r="C16" s="10" t="s">
-        <v>298</v>
       </c>
       <c r="D16" s="13" t="s">
         <v>152</v>
       </c>
       <c r="E16" s="10" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
     </row>
     <row r="17" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
+        <v>299</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>300</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="C17" s="5" t="s">
         <v>301</v>
-      </c>
-      <c r="C17" s="5" t="s">
-        <v>302</v>
       </c>
       <c r="D17" s="13" t="s">
         <v>152</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="37.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="9" t="s">
+        <v>303</v>
+      </c>
+      <c r="B18" s="10" t="s">
         <v>304</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="C18" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="D18" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="E18" s="10" t="s">
         <v>305</v>
-      </c>
-      <c r="C18" s="10" t="s">
-        <v>270</v>
-      </c>
-      <c r="D18" s="27" t="s">
-        <v>221</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="19" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
+        <v>306</v>
+      </c>
+      <c r="B19" s="5" t="s">
         <v>307</v>
       </c>
-      <c r="B19" s="5" t="s">
+      <c r="C19" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="D19" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="E19" s="5" t="s">
         <v>308</v>
-      </c>
-      <c r="C19" s="5" t="s">
-        <v>270</v>
-      </c>
-      <c r="D19" s="27" t="s">
-        <v>221</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>309</v>
       </c>
     </row>
     <row r="20" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="9" t="s">
+        <v>309</v>
+      </c>
+      <c r="B20" s="10" t="s">
         <v>310</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="C20" s="10" t="s">
+        <v>269</v>
+      </c>
+      <c r="D20" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="E20" s="10" t="s">
         <v>311</v>
-      </c>
-      <c r="C20" s="10" t="s">
-        <v>270</v>
-      </c>
-      <c r="D20" s="27" t="s">
-        <v>221</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="21" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
+        <v>312</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>313</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="C21" s="5" t="s">
         <v>314</v>
-      </c>
-      <c r="C21" s="5" t="s">
-        <v>315</v>
       </c>
       <c r="D21" s="11" t="s">
         <v>110</v>
@@ -3767,10 +3802,10 @@
     </row>
     <row r="22" spans="1:5" ht="37.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="9" t="s">
+        <v>315</v>
+      </c>
+      <c r="B22" s="10" t="s">
         <v>316</v>
-      </c>
-      <c r="B22" s="10" t="s">
-        <v>317</v>
       </c>
       <c r="C22" s="10" t="s">
         <v>115</v>
@@ -3779,49 +3814,49 @@
         <v>99</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
     </row>
     <row r="23" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
+        <v>317</v>
+      </c>
+      <c r="B23" s="5" t="s">
         <v>318</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="C23" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="D23" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="E23" s="5" t="s">
         <v>319</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>270</v>
-      </c>
-      <c r="D23" s="27" t="s">
-        <v>221</v>
-      </c>
-      <c r="E23" s="5" t="s">
-        <v>320</v>
       </c>
     </row>
     <row r="24" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="9" t="s">
+        <v>320</v>
+      </c>
+      <c r="B24" s="10" t="s">
         <v>321</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="C24" s="10" t="s">
         <v>322</v>
-      </c>
-      <c r="C24" s="10" t="s">
-        <v>323</v>
       </c>
       <c r="D24" s="13" t="s">
         <v>152</v>
       </c>
       <c r="E24" s="10" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
+        <v>324</v>
+      </c>
+      <c r="B25" s="5" t="s">
         <v>325</v>
-      </c>
-      <c r="B25" s="5" t="s">
-        <v>326</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>146</v>
@@ -3835,27 +3870,27 @@
     </row>
     <row r="26" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="9" t="s">
+        <v>326</v>
+      </c>
+      <c r="B26" s="10" t="s">
         <v>327</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="C26" s="10" t="s">
         <v>328</v>
-      </c>
-      <c r="C26" s="10" t="s">
-        <v>329</v>
       </c>
       <c r="D26" s="13" t="s">
         <v>152</v>
       </c>
       <c r="E26" s="10" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
     </row>
     <row r="27" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
+        <v>330</v>
+      </c>
+      <c r="B27" s="5" t="s">
         <v>331</v>
-      </c>
-      <c r="B27" s="5" t="s">
-        <v>332</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>167</v>
@@ -3864,15 +3899,15 @@
         <v>152</v>
       </c>
       <c r="E27" s="5" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
     </row>
     <row r="28" spans="1:5" ht="37.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="9" t="s">
+        <v>333</v>
+      </c>
+      <c r="B28" s="10" t="s">
         <v>334</v>
-      </c>
-      <c r="B28" s="10" t="s">
-        <v>335</v>
       </c>
       <c r="C28" s="10" t="s">
         <v>167</v>
@@ -3881,32 +3916,32 @@
         <v>152</v>
       </c>
       <c r="E28" s="10" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
     </row>
     <row r="29" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
+        <v>336</v>
+      </c>
+      <c r="B29" s="5" t="s">
         <v>337</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="C29" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="D29" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="E29" s="5" t="s">
         <v>338</v>
-      </c>
-      <c r="C29" s="5" t="s">
-        <v>270</v>
-      </c>
-      <c r="D29" s="27" t="s">
-        <v>221</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="30" spans="1:5" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="9" t="s">
+        <v>339</v>
+      </c>
+      <c r="B30" s="10" t="s">
         <v>340</v>
-      </c>
-      <c r="B30" s="10" t="s">
-        <v>341</v>
       </c>
       <c r="C30" s="10" t="s">
         <v>167</v>
@@ -3915,7 +3950,7 @@
         <v>152</v>
       </c>
       <c r="E30" s="10" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
     </row>
   </sheetData>
@@ -3947,7 +3982,7 @@
   <sheetData>
     <row r="1" spans="1:8" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="51" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="B1" s="35"/>
       <c r="C1" s="35"/>
@@ -3959,10 +3994,10 @@
     </row>
     <row r="2" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
+        <v>343</v>
+      </c>
+      <c r="B2" s="6" t="s">
         <v>344</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>345</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>76</v>
@@ -3974,13 +4009,13 @@
         <v>86</v>
       </c>
       <c r="F2" s="6" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="G2" s="6" t="s">
         <v>216</v>
       </c>
       <c r="H2" s="6" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="37.15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4032,7 +4067,7 @@
         <v>107</v>
       </c>
       <c r="H4" s="9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="37.15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4084,7 +4119,7 @@
         <v>107</v>
       </c>
       <c r="H6" s="9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="7" spans="1:8" ht="37.15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4110,7 +4145,7 @@
         <v>139</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="37.15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4136,7 +4171,7 @@
         <v>96</v>
       </c>
       <c r="H8" s="9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="37.15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4161,8 +4196,8 @@
       <c r="G9" s="5" t="s">
         <v>161</v>
       </c>
-      <c r="H9" s="7" t="s">
-        <v>221</v>
+      <c r="H9" s="53" t="s">
+        <v>353</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="37.15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4188,7 +4223,7 @@
         <v>161</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="37.15" customHeight="1" x14ac:dyDescent="0.25">
@@ -4292,7 +4327,7 @@
         <v>139</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
     </row>
   </sheetData>

</xml_diff>